<commit_message>
Point Colab setup at shared Drive folder BI10_ROUND01_DATASET
Accept transactions as either .parquet.gz or the .parquet/ CSV folder.
</commit_message>
<xml_diff>
--- a/draft/YAPPERS_huong_dan_Colab.xlsx
+++ b/draft/YAPPERS_huong_dan_Colab.xlsx
@@ -787,12 +787,12 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Tạo thư mục Google Drive BI10_YAPPERS_DATA, upload 3 file: consumer_financial_health_engagement_2025.csv (3MB), consumer_transactions_2025.parquet.gz (134MB), data_dictionary.xlsx</t>
+          <t>ĐÃ XONG: thư mục Drive BI10_ROUND01_DATASET https://drive.google.com/drive/folders/1gOqCyY9IfFUJtbr2r3vR_Z3t61O71CrC — cần có: consumer_financial_health_engagement_2025.csv (3MB), consumer_transactions_2025.parquet.gz (134MB), data_dictionary.xlsx</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Upload bản .parquet.gz (134MB) chứ KHÔNG phải CSV 597MB — setup tự giải nén. Share thư mục cho cả nhóm (Viewer).</t>
+          <t>File giao dịch: .parquet.gz hoặc thư mục .parquet/ chứa CSV đều được (setup tự xử lý). Share thư mục cho cả nhóm (Viewer).</t>
         </is>
       </c>
     </row>
@@ -807,12 +807,12 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Drive → 'Shared with me' → chuột phải BI10_YAPPERS_DATA → Organize → Add shortcut → My Drive</t>
+          <t>Drive → 'Shared with me' → chuột phải BI10_ROUND01_DATASET → Organize → Add shortcut → My Drive</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Để có đường dẫn /content/drive/MyDrive/BI10_YAPPERS_DATA. Leader thì thư mục đã nằm sẵn trong My Drive.</t>
+          <t>Để có đường dẫn /content/drive/MyDrive/BI10_ROUND01_DATASET. Leader thì thư mục đã nằm sẵn trong My Drive.</t>
         </is>
       </c>
     </row>
@@ -979,7 +979,7 @@
       <c r="B16" s="3" t="inlineStr"/>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>FileNotFoundError .../BI10_YAPPERS_DATA</t>
+          <t>FileNotFoundError .../BI10_ROUND01_DATASET</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Colab setup: download data from public Drive links, no mount needed
</commit_message>
<xml_diff>
--- a/draft/YAPPERS_huong_dan_Colab.xlsx
+++ b/draft/YAPPERS_huong_dan_Colab.xlsx
@@ -698,7 +698,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -787,12 +787,12 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>ĐÃ XONG: thư mục Drive BI10_ROUND01_DATASET https://drive.google.com/drive/folders/1gOqCyY9IfFUJtbr2r3vR_Z3t61O71CrC — cần có: consumer_financial_health_engagement_2025.csv (3MB), consumer_transactions_2025.parquet.gz (134MB), data_dictionary.xlsx</t>
+          <t>ĐÃ XONG: data ở thư mục Drive public https://drive.google.com/drive/folders/1gOqCyY9IfFUJtbr2r3vR_Z3t61O71CrC</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>File giao dịch: .parquet.gz hoặc thư mục .parquet/ chứa CSV đều được (setup tự xử lý). Share thư mục cho cả nhóm (Viewer).</t>
+          <t>Giữ quyền Anyone with the link. Cell SETUP tải thẳng bằng link — không cần mount Drive.</t>
         </is>
       </c>
     </row>
@@ -803,16 +803,16 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Drive → 'Shared with me' → chuột phải BI10_ROUND01_DATASET → Organize → Add shortcut → My Drive</t>
+          <t>GitHub → Settings → Developer settings → Personal access tokens → Fine-grained → repo BI10GroupYAPPERS, quyền Contents: Read</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Để có đường dẫn /content/drive/MyDrive/BI10_ROUND01_DATASET. Leader thì thư mục đã nằm sẵn trong My Drive.</t>
+          <t>Copy token (ghp_/github_pat_...).</t>
         </is>
       </c>
     </row>
@@ -823,18 +823,14 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>GitHub → Settings → Developer settings → Personal access tokens → Fine-grained → repo BI10GroupYAPPERS, quyền Contents: Read</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>Copy token (ghp_/github_pat_...).</t>
-        </is>
-      </c>
+          <t>Mở notebook của mình bằng link ở sheet 'Tổng quan' (lần đầu Colab xin quyền GitHub → cho phép, tick 'include private repos')</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -843,14 +839,18 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Mở notebook của mình bằng link ở sheet 'Tổng quan' (lần đầu Colab xin quyền GitHub → cho phép, tick 'include private repos')</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr"/>
+          <t>Colab → icon 🔑 (Secrets) bên trái → Add: Name = GH_TOKEN, Value = token → bật 'Notebook access'</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Token không nằm trong notebook → share không lộ.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -859,16 +859,16 @@
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Colab → icon 🔑 (Secrets) bên trái → Add: Name = GH_TOKEN, Value = token → bật 'Notebook access'</t>
+          <t>Runtime → Run all. Cell SETUP tự tải data (~1–2 phút)</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Token không nằm trong notebook → share không lộ.</t>
+          <t>Không cần pip install: Colab có sẵn pandas, numpy, sklearn, matplotlib, openpyxl.</t>
         </is>
       </c>
     </row>
@@ -879,16 +879,16 @@
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Runtime → Run all. Cell SETUP: cho phép mount Drive; chờ ~1 phút</t>
+          <t>Cell 'Bước 0' chạy script gốc → so với draft/taskN_output.txt</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Không cần pip install: Colab có sẵn pandas, numpy, sklearn, matplotlib, openpyxl.</t>
+          <t>Giống = setup đúng.</t>
         </is>
       </c>
     </row>
@@ -899,16 +899,16 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Cell 'Bước 0' chạy script gốc → so với draft/taskN_output.txt</t>
+          <t>Làm từng 'Việc' trong notebook; xong → File → Save a copy in GitHub → branch main, đúng path notebooks/&lt;file của mình&gt;</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Giống = setup đúng.</t>
+          <t>Mỗi người chỉ lưu notebook của mình → không conflict.</t>
         </is>
       </c>
     </row>
@@ -919,36 +919,34 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Làm từng 'Việc' trong notebook; xong → File → Save a copy in GitHub → branch main, đúng path notebooks/&lt;file của mình&gt;</t>
+          <t>Chart: savefig('outputs/figures/tN_ten.png') → tải về (thanh Files bên trái) → gửi P5</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Mỗi người chỉ lưu notebook của mình → không conflict.</t>
+          <t>outputs/ bị git-ignore.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Tất cả</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="n">
-        <v>11</v>
-      </c>
+          <t>Lỗi hay gặp</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr"/>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Chart: savefig('outputs/figures/tN_ten.png') → tải về (thanh Files bên trái) → gửi P5</t>
+          <t>Clone thất bại</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>outputs/ bị git-ignore.</t>
+          <t>Sai token / chưa được mời / chưa bật Notebook access cho GH_TOKEN.</t>
         </is>
       </c>
     </row>
@@ -961,12 +959,12 @@
       <c r="B15" s="3" t="inlineStr"/>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Clone thất bại</t>
+          <t>Lỗi tải (HTTP) / lỗi giải nén gzip</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Sai token / chưa được mời / chưa bật Notebook access cho GH_TOKEN.</t>
+          <t>Thư mục Drive bị tắt quyền Anyone with link, hoặc Drive giới hạn lượt tải → chờ vài phút rồi Run all lại.</t>
         </is>
       </c>
     </row>
@@ -979,28 +977,10 @@
       <c r="B16" s="3" t="inlineStr"/>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>FileNotFoundError .../BI10_ROUND01_DATASET</t>
+          <t>Runtime bị reset (sau ~90 phút idle)</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>Chưa Add shortcut vào My Drive, hoặc đặt tên thư mục khác → sửa biến DRIVE_DATA trong cell SETUP.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>Lỗi hay gặp</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr"/>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>Runtime bị reset (sau ~90 phút idle)</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
         <is>
           <t>Run all lại; data giải nén lại ~30s.</t>
         </is>

</xml_diff>

<commit_message>
Complete deep-dives for all 5 members and rebuild deck to 22 slides
- draft/taskN_deep.py (+ outputs): province channel mix, discretionary
  gradient, occupation groups, spend timing, crossover sensitivity,
  engagement heatmap, cutoff sensitivity, segment stability/migration,
  impact scenario
- notebooks: cells generated from the deep-dive scripts, findings filled
- findings: deep-dive sections; drop unsupported two-year caveat; fix
  digital value-share claim
- deck: 4 new slides, auto-numbered, updated exec summary and closing
</commit_message>
<xml_diff>
--- a/draft/YAPPERS_huong_dan_Colab.xlsx
+++ b/draft/YAPPERS_huong_dan_Colab.xlsx
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -666,6 +666,7 @@
         <v>7</v>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
@@ -698,7 +699,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1102,7 +1103,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
     </row>
@@ -1142,7 +1143,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
     </row>
@@ -1182,7 +1183,7 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
     </row>
@@ -1222,7 +1223,7 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
     </row>
@@ -1262,7 +1263,7 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
     </row>
@@ -1302,7 +1303,7 @@
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
     </row>
@@ -1428,7 +1429,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
     </row>
@@ -1468,7 +1469,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
     </row>
@@ -1509,7 +1510,7 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
     </row>
@@ -1549,7 +1550,7 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
     </row>
@@ -1674,7 +1675,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
     </row>
@@ -1714,7 +1715,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
     </row>
@@ -1754,7 +1755,7 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
     </row>
@@ -1794,7 +1795,7 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
     </row>
@@ -1834,7 +1835,7 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
     </row>
@@ -1874,7 +1875,7 @@
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1915,7 @@
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đang làm</t>
         </is>
       </c>
     </row>
@@ -2039,7 +2040,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
     </row>
@@ -2080,7 +2081,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
     </row>
@@ -2120,7 +2121,7 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
     </row>
@@ -2160,7 +2161,7 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
     </row>
@@ -2200,7 +2201,7 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
     </row>
@@ -2240,7 +2241,7 @@
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
     </row>
@@ -2365,7 +2366,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đang làm</t>
         </is>
       </c>
     </row>
@@ -2405,7 +2406,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
     </row>
@@ -2445,7 +2446,7 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
     </row>
@@ -2485,7 +2486,7 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đang làm</t>
         </is>
       </c>
     </row>
@@ -2526,7 +2527,7 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
     </row>
@@ -2566,7 +2567,7 @@
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đang làm</t>
         </is>
       </c>
     </row>
@@ -2606,7 +2607,7 @@
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đang làm</t>
         </is>
       </c>
     </row>
@@ -2626,7 +2627,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2788,7 +2789,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>

</xml_diff>

<commit_message>
Add full_pipeline notebook (tasks 1-5 + charts); token prompt fallback; classic-token guide
</commit_message>
<xml_diff>
--- a/draft/YAPPERS_huong_dan_Colab.xlsx
+++ b/draft/YAPPERS_huong_dan_Colab.xlsx
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -666,7 +666,6 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
@@ -678,6 +677,18 @@
       <c r="A11" s="5" t="inlineStr">
         <is>
           <t>Quy tắc sửa file: mỗi người chỉ sửa notebook + findings của mình; build_deck.js / .pptx chỉ P5. Đổi con số nào → báo P5 ngay.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Notebook tổng (chạy cả 5 task + vẽ lại toàn bộ chart):</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>https://colab.research.google.com/github/thanh-tai-435/BI10GroupYAPPERS/blob/main/notebooks/full_pipeline.ipynb</t>
         </is>
       </c>
     </row>
@@ -688,6 +699,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -699,7 +711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -748,7 +760,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Push code lên GitHub (hiện repo trên GitHub mới chỉ có scaffold, chưa có draft/ + notebooks/)</t>
+          <t>ĐÃ XONG: code, notebook, deck đã push lên GitHub (main).</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -808,12 +820,12 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>GitHub → Settings → Developer settings → Personal access tokens → Fine-grained → repo BI10GroupYAPPERS, quyền Contents: Read</t>
+          <t>Mở https://github.com/settings/tokens/new (Tokens CLASSIC) → Note: colab-yappers · Expiration: 7 days · tick scope "repo" → Generate token → copy ghp_... (chỉ hiện 1 lần)</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Copy token (ghp_/github_pat_...).</t>
+          <t>Phải chấp nhận lời mời vào repo trước. KHÔNG dùng Fine-grained: không truy cập được repo cá nhân của người khác khi chỉ là collaborator.</t>
         </is>
       </c>
     </row>
@@ -849,7 +861,7 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Token không nằm trong notebook → share không lộ.</t>
+          <t>Token không nằm trong notebook → share không lộ. Bỏ qua bước này cũng được: cell SETUP sẽ hiện ô để dán token.</t>
         </is>
       </c>
     </row>
@@ -2627,7 +2639,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2789,7 +2801,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>

</xml_diff>